<commit_message>
Add basin summary QA checks, standardised naming, and improved output file structure
</commit_message>
<xml_diff>
--- a/check_outputs/fu_all_regions/fu_report_qa.xlsx
+++ b/check_outputs/fu_all_regions/fu_report_qa.xlsx
@@ -416,31 +416,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>FU</t>
+          <t>FS</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>FS</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PP</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
-        <is>
-          <t>PP</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
         <is>
           <t>DIN</t>
         </is>
@@ -457,153 +452,98 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>FU</t>
+          <t>max_abs_difference</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>max_abs_difference</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
           <t>within_tolerance</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Bananas</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" t="b">
+      <c r="A2" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Conservation</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C3" t="b">
+      <c r="A3" t="n">
+        <v>0</v>
+      </c>
+      <c r="B3" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Cropping</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" t="b">
+      <c r="A4" t="n">
+        <v>0</v>
+      </c>
+      <c r="B4" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Dairy</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" t="b">
+      <c r="A5" t="n">
+        <v>0</v>
+      </c>
+      <c r="B5" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Forestry</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" t="b">
+      <c r="A6" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Grazing</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" t="b">
+      <c r="A7" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Horticulture</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" t="b">
+      <c r="A8" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Stream</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" t="b">
+      <c r="A9" t="n">
+        <v>0</v>
+      </c>
+      <c r="B9" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Sugarcane</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" t="b">
+      <c r="A10" t="n">
+        <v>0</v>
+      </c>
+      <c r="B10" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Urban + Other</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" t="b">
+      <c r="A11" t="n">
+        <v>0</v>
+      </c>
+      <c r="B11" t="b">
         <v>1</v>
       </c>
     </row>
@@ -618,153 +558,98 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>FU</t>
+          <t>max_abs_difference</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>max_abs_difference</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
           <t>within_tolerance</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Bananas</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" t="b">
+      <c r="A2" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Conservation</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C3" t="b">
+      <c r="A3" t="n">
+        <v>0</v>
+      </c>
+      <c r="B3" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Cropping</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" t="b">
+      <c r="A4" t="n">
+        <v>0</v>
+      </c>
+      <c r="B4" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Dairy</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" t="b">
+      <c r="A5" t="n">
+        <v>0</v>
+      </c>
+      <c r="B5" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Forestry</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" t="b">
+      <c r="A6" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Grazing</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" t="b">
+      <c r="A7" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Horticulture</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" t="b">
+      <c r="A8" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Stream</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" t="b">
+      <c r="A9" t="n">
+        <v>0</v>
+      </c>
+      <c r="B9" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Sugarcane</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" t="b">
+      <c r="A10" t="n">
+        <v>0</v>
+      </c>
+      <c r="B10" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Urban + Other</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" t="b">
+      <c r="A11" t="n">
+        <v>0</v>
+      </c>
+      <c r="B11" t="b">
         <v>1</v>
       </c>
     </row>
@@ -779,31 +664,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>FU</t>
+          <t>FS</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>FS</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PP</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
-        <is>
-          <t>PP</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
         <is>
           <t>DIN</t>
         </is>

</xml_diff>